<commit_message>
GBDS JUNE FILES 2026 } berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JUNE FILES 2026/PURCHASES - JUNE 2026.xlsx
+++ b/GBDS JUNE FILES 2026/PURCHASES - JUNE 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JUNE FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDD7DA3-2954-4E2A-B04A-F13B835476F1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FCFB00-7B70-4E18-89D0-94AE4D022715}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="420" windowWidth="29040" windowHeight="15900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE" sheetId="4" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="80">
   <si>
     <t>HOME MART ENTERPRISES</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>06/19/2026</t>
+  </si>
+  <si>
+    <t>06/23/2026</t>
   </si>
 </sst>
 </file>
@@ -2508,7 +2511,9 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="C10" s="19"/>
+      <c r="C10" s="19" t="s">
+        <v>79</v>
+      </c>
       <c r="D10" s="20" t="s">
         <v>68</v>
       </c>
@@ -2516,22 +2521,27 @@
       <c r="F10" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="20"/>
+      <c r="G10" s="20">
+        <v>518756120</v>
+      </c>
       <c r="H10" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="21"/>
+      <c r="I10" s="21">
+        <f>1346606-57095.42</f>
+        <v>1289510.58</v>
+      </c>
       <c r="K10" s="21">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>138161.84785714286</v>
       </c>
       <c r="L10" s="27">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1151348.7321428573</v>
       </c>
       <c r="M10" s="33">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>11513.487321428573</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -3157,20 +3167,20 @@
       <c r="G32"/>
       <c r="I32" s="46">
         <f>SUM(I7:I31)</f>
-        <v>3729565.66</v>
+        <v>5019076.24</v>
       </c>
       <c r="J32" s="47"/>
       <c r="K32" s="46">
         <f>SUM(K7:K31)</f>
-        <v>399596.32071428571</v>
+        <v>537758.16857142863</v>
       </c>
       <c r="L32" s="46">
         <f>SUM(L7:L31)</f>
-        <v>3329969.3392857146</v>
+        <v>4481318.0714285718</v>
       </c>
       <c r="M32" s="48">
         <f>SUM(M7:M31)</f>
-        <v>33299.693392857145</v>
+        <v>44813.180714285714</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>